<commit_message>
add list example 1d188bf031e1bb207af969e3588ffc61b6f74f22
</commit_message>
<xml_diff>
--- a/nr-add-examples/ig/StructureDefinition-pdsm-folder-comprehensive.xlsx
+++ b/nr-add-examples/ig/StructureDefinition-pdsm-folder-comprehensive.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-04-30T07:39:59+00:00</t>
+    <t>2025-04-30T07:55:10+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -84,7 +84,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Profil spécifique dérivé du profil IHE MHD « Comprehensive Folder » créé pour le volet ANS "Partage de documents de santé en mobilité" ; ce profil concerne le classeur.</t>
+    <t>Profil du Classeur dérivé de la ressource List et du profil IHE MHD « Comprehensive Folder ».</t>
   </si>
   <si>
     <t>Purpose</t>

</xml_diff>